<commit_message>
Update DWEC submodule reference and add dirty flag to the commit
</commit_message>
<xml_diff>
--- a/asignaturas/BI/EXCEL/04 octubre/4 de Octubre.xlsx
+++ b/asignaturas/BI/EXCEL/04 octubre/4 de Octubre.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DAW\asignaturas\BI\EXCEL\04 octubre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E894ED7-3FE7-4CDB-AD3A-F221F41956C9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{677989F5-D14C-43E9-966B-F2ACD64D375A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ejercicio contar" sheetId="2" r:id="rId1"/>
-    <sheet name="Ejercicio conjunto" sheetId="1" r:id="rId2"/>
+    <sheet name="Hoja1" sheetId="3" r:id="rId2"/>
+    <sheet name="Ejercicio conjunto" sheetId="1" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="70">
   <si>
     <t>Comercial</t>
   </si>
@@ -212,6 +213,30 @@
   </si>
   <si>
     <t>1)CUANTOS VENDEDORES TIENEN VENTAS?</t>
+  </si>
+  <si>
+    <t>par</t>
+  </si>
+  <si>
+    <t>ciudad</t>
+  </si>
+  <si>
+    <t>telefono</t>
+  </si>
+  <si>
+    <t>edad</t>
+  </si>
+  <si>
+    <t>nombre</t>
+  </si>
+  <si>
+    <t>madrid</t>
+  </si>
+  <si>
+    <t>toledo</t>
+  </si>
+  <si>
+    <t>observaciones</t>
   </si>
 </sst>
 </file>
@@ -1034,7 +1059,7 @@
       <c r="D17" s="17"/>
       <c r="E17" s="17"/>
       <c r="F17" s="11">
-        <f t="shared" ref="F14:F21" si="0">COUNT(E8:E15)</f>
+        <f t="shared" ref="F17" si="0">COUNT(E8:E15)</f>
         <v>4</v>
       </c>
     </row>
@@ -1145,6 +1170,74 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC370157-9A88-4226-8A93-026010CF5802}">
+  <dimension ref="B4:G8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="7" max="7" width="13.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D4" t="s">
+        <v>65</v>
+      </c>
+      <c r="E4" t="s">
+        <v>64</v>
+      </c>
+      <c r="F4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="F5" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B6">
+        <v>6</v>
+      </c>
+      <c r="D6">
+        <v>19</v>
+      </c>
+      <c r="E6">
+        <v>987456321</v>
+      </c>
+      <c r="F6" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D7">
+        <v>18</v>
+      </c>
+      <c r="E7">
+        <v>65505779</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B8">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B1:L26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>